<commit_message>
feat(templates): add Dimensions / Size, Table Top Finish / Wood, and Leg Type / Color explicit columns to bulk upload Excel and CSV templates
</commit_message>
<xml_diff>
--- a/public/templates/bosq_master_product_bulk_import_template.xlsx
+++ b/public/templates/bosq_master_product_bulk_import_template.xlsx
@@ -39,10 +39,10 @@
     <t>Chair Type</t>
   </si>
   <si>
-    <t>Table Top Finish</t>
-  </si>
-  <si>
-    <t>Leg Type</t>
+    <t>Table Top Finish / Wood</t>
+  </si>
+  <si>
+    <t>Leg Type / Color</t>
   </si>
   <si>
     <t>Storage Options</t>
@@ -51,7 +51,7 @@
     <t>Finish Material</t>
   </si>
   <si>
-    <t>Dimensions</t>
+    <t>Dimensions / Size</t>
   </si>
   <si>
     <t>Product Description</t>
@@ -862,7 +862,8 @@
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="10" width="22" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
     <col min="11" max="11" width="24" customWidth="1"/>
     <col min="12" max="12" width="22" customWidth="1"/>
     <col min="13" max="13" width="24" customWidth="1"/>

</xml_diff>